<commit_message>
docs: add comprehensive manual UAT guide for Google integration and update test specifications to pending manual verification
</commit_message>
<xml_diff>
--- a/docs/GoogleDrive_Upload/Mauro_Brenda_Taxi_Link_シナリオテスト仕様書.xlsx
+++ b/docs/GoogleDrive_Upload/Mauro_Brenda_Taxi_Link_シナリオテスト仕様書.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="テスト概要・サマリー" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="受入テスト結果・証跡一覧" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="シナリオテストケース一覧" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Google連携手動受入検証手順" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,13 +63,37 @@
       <sz val="10"/>
     </font>
     <font>
+      <name val="Meiryo"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <name val="Consolas"/>
       <b val="1"/>
       <color rgb="000284C7"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Meiryo"/>
+      <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Meiryo"/>
+      <b val="1"/>
+      <color rgb="000284C7"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Meiryo"/>
+      <b val="1"/>
+      <color rgb="00059669"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -95,6 +120,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -147,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -160,38 +191,85 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -557,11 +635,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G25"/>
+  <dimension ref="B2:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="75" customWidth="1" min="3" max="3"/>
+    <col width="85" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -574,7 +652,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>受入シナリオテスト仕様書 ＆ 全項目客観的証跡（キャプチャー・ログ）報告書</t>
+          <t>受入シナリオテスト仕様書 ＆ 手動受入検証管理表</t>
         </is>
       </c>
     </row>
@@ -634,164 +712,200 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>全28テストケースの自動E2Eブラウザ実行、DOM検証、および客観的証跡（全項目画面キャプチャー・全行ログ）の採取</t>
+          <t>全28シナリオの受入検証（Web自動E2E検証 22件 ＋ 本番Google手動連携検証 6件）</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>テスト実施環境</t>
+          <t>Web自動E2E検証</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Puppeteer (Chromium Headless / 1280x800 PC &amp; 375x812 スマホ)</t>
+          <t>22項目 実施完了 / PASS: 22件, FAIL: 0件 (合格率 100% / 客観的証跡画像22枚+ログ完備)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>テスト実施日</t>
+          <t>Google連携手動検証</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>2026年10月08日</t>
+          <t>6項目 / ステータス: 【手動受入検証待ち】（非技術者向け手順書に基づき本番アカウントで実施・証跡取得後に正式合格）</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>テスト実行結果</t>
+          <t>総合判定ルール</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>全28項目 実施完了 / PASS: 28件, FAIL: 0件 (合格率 100%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>証跡ファイル保存先</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>docs/evidence/ (全28画像 + test_execution_log.txt)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>総合判定</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>合格 (Pass) - 全項目に実行ログおよびキャプチャー証跡を完備</t>
+          <t>Web基本機能は完全動作確認済。Google実機連携はユーザー手動確認の証跡取得をもって最終合格・本番承認とする</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>カテゴリ別 テスト検証状況</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>カテゴリ別 テスト実行・証跡取得集計</t>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>カテゴリ</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>対象機能</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>ケース数</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>検証方式</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>証跡状況</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>判定ステータス</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>1. 保護者ポータル</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>生徒切替・残高確認・アラート・予約・自己キャンセル・履歴閲覧</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Puppeteer E2E自動</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>画面キャプチャー9枚 + ログ</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>OK (PASS 100%)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>カテゴリ</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>対象機能</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>ケース数</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>E2E実行</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>証跡画像数</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>判定</t>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>2. 管理者ダッシュボード</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>サマリー・送迎完了減算・地図連動・予定追加・生徒登録・チャージ・取消</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Puppeteer E2E自動</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>画面キャプチャー8枚 + ログ</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>OK (PASS 100%)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>1. 保護者ポータル</t>
+          <t>3. データ整合性</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>生徒切替・残高確認・アラート・予約・自己キャンセル・履歴閲覧</t>
+          <t>予約〜完了往復連携・残数0境界値警告・リロード永続化</t>
         </is>
       </c>
       <c r="D20" s="7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>E2E自動実行済</t>
+          <t>Puppeteer E2E自動</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>9枚</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
+          <t>画面キャプチャー3枚 + ログ</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>OK (PASS 100%)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>2. 管理者ダッシュボード</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>サマリー・送迎完了減算・地図連動・予定追加・生徒登録・チャージ・取消</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>E2E自動実行済</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>8枚</t>
-        </is>
-      </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>4. デザイン＆レスポンシブ</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>スマートフォン(375px)適合・全画面ビジュアル品質</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Puppeteer E2E自動</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>画面キャプチャー2枚 + ログ</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
         <is>
           <t>OK (PASS 100%)</t>
         </is>
@@ -800,120 +914,60 @@
     <row r="22">
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>3. データ整合性</t>
+          <t>5. Google連携 (GAS)</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>予約〜完了往復連携・残数0境界値警告・リロード永続化</t>
+          <t>シート自動初期化・URL設定・カレンダー同期/削除・フォールバック</t>
         </is>
       </c>
       <c r="D22" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>E2E自動実行済</t>
+          <t>手動受入検証 (UAT)</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>3枚</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>OK (PASS 100%)</t>
+          <t>手動実施時の実画面キャプチャー4枚で判定</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>手動受入検証待ち</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>4. Google連携 (GAS)</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>コード表示コピー・シート初期化・URL設定保存・カレンダー同期/削除・フォールバック</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>E2E自動実行済</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>6枚</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>OK (PASS 100%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>5. デザイン＆レスポンシブ</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>スマートフォン(375px)適合・全画面ビジュアル品質</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>E2E自動実行済</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>2枚</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>OK (PASS 100%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
         <is>
           <t>全機能完全網羅</t>
         </is>
       </c>
-      <c r="D25" s="11" t="n">
+      <c r="D23" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>全件完全実行</t>
-        </is>
-      </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>28枚</t>
-        </is>
-      </c>
-      <c r="G25" s="11" t="inlineStr">
-        <is>
-          <t>OK (全件合格)</t>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>自動22件 ＋ 手動6件</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>自動22枚完備 ＋ 手動4枚予定</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>22件合格 / 6件手動確認中</t>
         </is>
       </c>
     </row>
@@ -934,1610 +988,1879 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>テストID</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>カテゴリ</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>テストケース名</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>前提条件</t>
         </is>
       </c>
-      <c r="F2" s="12" t="inlineStr">
+      <c r="F2" s="15" t="inlineStr">
         <is>
           <t>操作手順</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="G2" s="15" t="inlineStr">
         <is>
           <t>期待される結果（合格基準）</t>
         </is>
       </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="H2" s="15" t="inlineStr">
         <is>
           <t>判定</t>
         </is>
       </c>
-      <c r="I2" s="12" t="inlineStr">
-        <is>
-          <t>実施方式</t>
-        </is>
-      </c>
-      <c r="J2" s="12" t="inlineStr">
-        <is>
-          <t>証跡画像ファイル</t>
-        </is>
-      </c>
-      <c r="K2" s="12" t="inlineStr">
-        <is>
-          <t>E2E実行ログ・証跡詳細</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="13" t="n">
+      <c r="I2" s="15" t="inlineStr">
+        <is>
+          <t>検証方式</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>証跡状況 / ファイル名</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="inlineStr">
+        <is>
+          <t>実行ログ・受入確認詳細</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>TC-P01</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>送迎利用者</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>生徒切り替え操作</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>複数生徒が登録されている</t>
         </is>
       </c>
-      <c r="F3" s="14" t="inlineStr">
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>画面上部「表示する生徒」プルダウンから別生徒を選択</t>
         </is>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>選択生徒の残高・予約一覧・過去履歴が即座に同期切り替えされる</t>
         </is>
       </c>
-      <c r="H3" s="15" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I3" s="13" t="inlineStr">
+      <c r="I3" s="16" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J3" s="16" t="inlineStr">
+      <c r="J3" s="19" t="inlineStr">
         <is>
           <t>TC-P01_student_switch.png</t>
         </is>
       </c>
-      <c r="K3" s="14" t="inlineStr">
+      <c r="K3" s="17" t="inlineStr">
         <is>
           <t>生徒「山本 颯太」へ切り替え成功。残1回表示と予約一覧の同期を確認。</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="17" t="n">
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>TC-P02</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>送迎利用者</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>チケット残数表示（余裕時）</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>チケット残3回以上</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>保護者ポータルを開く</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G4" s="21" t="inlineStr">
         <is>
           <t>残回数が大きく表示され「片道1枚消費」が明記。警告枠は非表示</t>
         </is>
       </c>
-      <c r="H4" s="15" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I4" s="17" t="inlineStr">
+      <c r="I4" s="20" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
+      <c r="J4" s="22" t="inlineStr">
         <is>
           <t>TC-P02_residual_normal.png</t>
         </is>
       </c>
-      <c r="K4" s="18" t="inlineStr">
+      <c r="K4" s="21" t="inlineStr">
         <is>
           <t>田中 陽菜さん 残7回分および「片道1回につきチケット1枚消費」表示を確認。</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="13" t="n">
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>TC-P03</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>送迎利用者</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>残少アラート表示（残り1回）</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>チケット残2回以下</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>山本 颯太さん（残1回）を選択</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>「⚠️ チケットが無くなりそうです（残り1回）Mauro・Brenda に連絡してね！」が表示される</t>
         </is>
       </c>
-      <c r="H5" s="15" t="inlineStr">
+      <c r="H5" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
+      <c r="I5" s="16" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J5" s="16" t="inlineStr">
+      <c r="J5" s="19" t="inlineStr">
         <is>
           <t>TC-P03_residual_alert.png</t>
         </is>
       </c>
-      <c r="K5" s="14" t="inlineStr">
+      <c r="K5" s="17" t="inlineStr">
         <is>
           <t>警告枠および指定メッセージの完全一致レンダリングを確認。</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="17" t="n">
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>TC-P04</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>送迎利用者</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>チケット残ゼロ表示</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>チケット残0回</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F6" s="21" t="inlineStr">
         <is>
           <t>高橋 莉子さん（残0回）を選択</t>
         </is>
       </c>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="G6" s="21" t="inlineStr">
         <is>
           <t>残高0回分と表示され、警告アラートが表示される</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="H6" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I6" s="17" t="inlineStr">
+      <c r="I6" s="20" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J6" s="19" t="inlineStr">
+      <c r="J6" s="22" t="inlineStr">
         <is>
           <t>TC-P04_residual_zero.png</t>
         </is>
       </c>
-      <c r="K6" s="18" t="inlineStr">
+      <c r="K6" s="21" t="inlineStr">
         <is>
           <t>高橋 莉子さん 残0回分表示および警告枠を確認。</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="13" t="n">
+    <row r="7" ht="25" customHeight="1">
+      <c r="A7" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>TC-P05</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>送迎利用者</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>送迎予約登録（行き・お迎え）</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>残チケット1枚以上</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>予約モーダルで「行き（お迎え）」を選択し確定</t>
         </is>
       </c>
-      <c r="G7" s="14" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr">
         <is>
           <t>予約一覧に「お迎え（教室へ）」で登録。確定時点では残数減算なし</t>
         </is>
       </c>
-      <c r="H7" s="15" t="inlineStr">
+      <c r="H7" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I7" s="13" t="inlineStr">
+      <c r="I7" s="16" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J7" s="16" t="inlineStr">
+      <c r="J7" s="19" t="inlineStr">
         <is>
           <t>TC-P05_reservation_pickup.png</t>
         </is>
       </c>
-      <c r="K7" s="14" t="inlineStr">
+      <c r="K7" s="17" t="inlineStr">
         <is>
           <t>「お迎え（教室へ）」送迎予約の新規登録・一覧反映を確認。</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="17" t="n">
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>TC-P06</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>送迎利用者</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>送迎予約登録（帰り・送り）</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>残チケット1枚以上</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F8" s="21" t="inlineStr">
         <is>
           <t>予約モーダルで「帰り（送り）」を選択し確定</t>
         </is>
       </c>
-      <c r="G8" s="18" t="inlineStr">
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>予約一覧に「送り（ご自宅へ）」で正常に登録される</t>
         </is>
       </c>
-      <c r="H8" s="15" t="inlineStr">
+      <c r="H8" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I8" s="17" t="inlineStr">
+      <c r="I8" s="20" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J8" s="19" t="inlineStr">
+      <c r="J8" s="22" t="inlineStr">
         <is>
           <t>TC-P06_reservation_dropoff.png</t>
         </is>
       </c>
-      <c r="K8" s="18" t="inlineStr">
+      <c r="K8" s="21" t="inlineStr">
         <is>
           <t>「送り（ご自宅へ）」送迎予約の新規登録・一覧反映を確認。</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="13" t="n">
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>TC-P07</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>送迎利用者</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>送迎予約登録（往復・2枚消費）</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>残チケット2枚以上</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>予約モーダルで「往復」を選択し確定</t>
         </is>
       </c>
-      <c r="G9" s="14" t="inlineStr">
+      <c r="G9" s="17" t="inlineStr">
         <is>
           <t>「往復（チケット2枚消費）」の明記とともに正常登録される</t>
         </is>
       </c>
-      <c r="H9" s="15" t="inlineStr">
+      <c r="H9" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I9" s="13" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J9" s="16" t="inlineStr">
+      <c r="J9" s="19" t="inlineStr">
         <is>
           <t>TC-P07_reservation_roundtrip.png</t>
         </is>
       </c>
-      <c r="K9" s="14" t="inlineStr">
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>「往復」送迎予約（チケット2枚消費）の登録成功を確認。</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="17" t="n">
+    <row r="10" ht="25" customHeight="1">
+      <c r="A10" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>TC-P08</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>送迎利用者</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>保護者による自己キャンセル</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>予約中データが存在する</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="21" t="inlineStr">
         <is>
           <t>予約の「キャンセル」をクリックしダイアログOK</t>
         </is>
       </c>
-      <c r="G10" s="18" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>予約中から消え、過去履歴に「キャンセル」で記録。残数は減らない</t>
         </is>
       </c>
-      <c r="H10" s="15" t="inlineStr">
+      <c r="H10" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I10" s="17" t="inlineStr">
+      <c r="I10" s="20" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J10" s="19" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>TC-P08_reservation_cancel.png</t>
         </is>
       </c>
-      <c r="K10" s="18" t="inlineStr">
+      <c r="K10" s="21" t="inlineStr">
         <is>
           <t>送迎予定のキャンセル実行および過去履歴への「キャンセル」移動を確認（confirm自動承諾）。</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="13" t="n">
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>TC-P09</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>送迎利用者</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>過去利用履歴テーブル閲覧</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>完了・キャンセルデータあり</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>ポータル下部の過去履歴テーブルを確認</t>
         </is>
       </c>
-      <c r="G11" s="14" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>日時・種別・ステータス（送迎済 / キャンセル）が時系列表示される</t>
         </is>
       </c>
-      <c r="H11" s="15" t="inlineStr">
+      <c r="H11" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I11" s="13" t="inlineStr">
+      <c r="I11" s="16" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J11" s="16" t="inlineStr">
+      <c r="J11" s="19" t="inlineStr">
         <is>
           <t>TC-P09_history_table.png</t>
         </is>
       </c>
-      <c r="K11" s="14" t="inlineStr">
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>過去の送迎実績・ステータス（送迎済 / キャンセル）が履歴表に正確に表示されていることを確認。</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="17" t="n">
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>TC-T01</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>管理者</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>管理者ダッシュボード＆サマリー</t>
         </is>
       </c>
-      <c r="E12" s="18" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
         <is>
           <t>当日予定が存在する</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="F12" s="21" t="inlineStr">
         <is>
           <t>「管理者用」タブを選択</t>
         </is>
       </c>
-      <c r="G12" s="18" t="inlineStr">
+      <c r="G12" s="21" t="inlineStr">
         <is>
           <t>バナー表示、本日の件数サマリー、チケット残少生徒数が正確に集計表示</t>
         </is>
       </c>
-      <c r="H12" s="15" t="inlineStr">
+      <c r="H12" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I12" s="17" t="inlineStr">
+      <c r="I12" s="20" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J12" s="19" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>TC-T01_teacher_summary.png</t>
         </is>
       </c>
-      <c r="K12" s="18" t="inlineStr">
+      <c r="K12" s="21" t="inlineStr">
         <is>
           <t>「Mauro・Brenda 先生用管理ダッシュボード」バナーおよび3カードサマリーを確認。</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="13" t="n">
+    <row r="13" ht="25" customHeight="1">
+      <c r="A13" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>TC-T02</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>管理者</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>送迎完了処理とチケット自動減算</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>当日予定が未完了(scheduled)</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr">
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>送迎カードの「送迎完了（1回消費）」をクリック</t>
         </is>
       </c>
-      <c r="G13" s="14" t="inlineStr">
+      <c r="G13" s="17" t="inlineStr">
         <is>
           <t>カードが完了状態になり、該当生徒のチケット残高が即座に-1減算される</t>
         </is>
       </c>
-      <c r="H13" s="15" t="inlineStr">
+      <c r="H13" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I13" s="13" t="inlineStr">
+      <c r="I13" s="16" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J13" s="16" t="inlineStr">
+      <c r="J13" s="19" t="inlineStr">
         <is>
           <t>TC-T02_ride_completed.png</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
+      <c r="K13" s="17" t="inlineStr">
         <is>
           <t>送迎完了処理を実行し、チケットが自動で-1枚減算されステータスが更新されたことを確認。</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="17" t="n">
+    <row r="14" ht="25" customHeight="1">
+      <c r="A14" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>TC-T03</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>管理者</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>Google Maps地図アプリ連動</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>送迎先住所あり</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F14" s="21" t="inlineStr">
         <is>
           <t>カード内の「地図アプリ」をクリック</t>
         </is>
       </c>
-      <c r="G14" s="18" t="inlineStr">
+      <c r="G14" s="21" t="inlineStr">
         <is>
           <t>Google Mapsが新規タブで開き、送迎先住所がピン留め検索される</t>
         </is>
       </c>
-      <c r="H14" s="15" t="inlineStr">
+      <c r="H14" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I14" s="17" t="inlineStr">
+      <c r="I14" s="20" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J14" s="19" t="inlineStr">
+      <c r="J14" s="22" t="inlineStr">
         <is>
           <t>TC-T03_map_link.png</t>
         </is>
       </c>
-      <c r="K14" s="18" t="inlineStr">
-        <is>
-          <t>地図アプリボタンがGoogle Maps検索リンク（maps/search/?api=1&amp;query=...）と連携していることを確認。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="13" t="n">
+      <c r="K14" s="21" t="inlineStr">
+        <is>
+          <t>地図アプリボタンがGoogle Maps検索リンクと連携していることを確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="25" customHeight="1">
+      <c r="A15" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>TC-T04</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>管理者</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>先生側からの送迎予定追加</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F15" s="14" t="inlineStr">
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>「送迎予定を追加」より生徒・日時・区分を入力</t>
         </is>
       </c>
-      <c r="G15" s="14" t="inlineStr">
+      <c r="G15" s="17" t="inlineStr">
         <is>
           <t>一覧および全スケジュールに即座反映。生徒選択で登録住所が自動補完</t>
         </is>
       </c>
-      <c r="H15" s="15" t="inlineStr">
+      <c r="H15" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I15" s="13" t="inlineStr">
+      <c r="I15" s="16" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J15" s="16" t="inlineStr">
+      <c r="J15" s="19" t="inlineStr">
         <is>
           <t>TC-T04_teacher_add_ride.png</t>
         </is>
       </c>
-      <c r="K15" s="14" t="inlineStr">
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>先生用画面からの送迎予定追加モーダルおよびスケジュール反映を確認。</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="17" t="n">
+    <row r="16" ht="25" customHeight="1">
+      <c r="A16" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="17" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>TC-T05</t>
         </is>
       </c>
-      <c r="C16" s="17" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>管理者</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>新規生徒登録（住所・連絡先含む）</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F16" s="21" t="inlineStr">
         <is>
           <t>生徒管理タブで「＋新規生徒を登録」をクリックし保存</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>生徒一覧および保護者ポータルのプルダウンに新規生徒が即時追加される</t>
         </is>
       </c>
-      <c r="H16" s="15" t="inlineStr">
+      <c r="H16" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I16" s="17" t="inlineStr">
+      <c r="I16" s="20" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J16" s="19" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>TC-T05_add_student.png</t>
         </is>
       </c>
-      <c r="K16" s="18" t="inlineStr">
+      <c r="K16" s="21" t="inlineStr">
         <is>
           <t>新規生徒「鈴木 陸斗」の登録実行および台帳一覧への即時追加を確認。</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="13" t="n">
+    <row r="17" ht="25" customHeight="1">
+      <c r="A17" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>TC-T06</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="16" t="inlineStr">
         <is>
           <t>管理者</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>チケット追加チャージ（10回券）</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="F17" s="17" t="inlineStr">
         <is>
           <t>「チケット追加」より10回券(¥10,000)を選択して登録</t>
         </is>
       </c>
-      <c r="G17" s="14" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>生徒のチケット残数が+10され、残少だった場合はアラートが自動解除</t>
         </is>
       </c>
-      <c r="H17" s="15" t="inlineStr">
+      <c r="H17" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I17" s="13" t="inlineStr">
+      <c r="I17" s="16" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J17" s="16" t="inlineStr">
+      <c r="J17" s="19" t="inlineStr">
         <is>
           <t>TC-T06_add_ticket.png</t>
         </is>
       </c>
-      <c r="K17" s="14" t="inlineStr">
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t>10回券（+10回分）のチャージ処理成功および生徒残数加算を確認。</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="17" t="n">
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>TC-T07</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>管理者</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>送迎スケジュール一覧と絞り込み</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E18" s="21" t="inlineStr">
         <is>
           <t>複数送迎データあり</t>
         </is>
       </c>
-      <c r="F18" s="18" t="inlineStr">
+      <c r="F18" s="21" t="inlineStr">
         <is>
           <t>スケジュール一覧で「予約中」「完了済み」「キャンセル」を切り替え</t>
         </is>
       </c>
-      <c r="G18" s="18" t="inlineStr">
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>選択したステータスに合致する送迎データのみが正確に一覧表示される</t>
         </is>
       </c>
-      <c r="H18" s="15" t="inlineStr">
+      <c r="H18" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I18" s="17" t="inlineStr">
+      <c r="I18" s="20" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J18" s="19" t="inlineStr">
+      <c r="J18" s="22" t="inlineStr">
         <is>
           <t>TC-T07_schedule_filter.png</t>
         </is>
       </c>
-      <c r="K18" s="18" t="inlineStr">
+      <c r="K18" s="21" t="inlineStr">
         <is>
           <t>スケジュール一覧におけるステータスフィルター（完了済み）による絞り込み表示を確認。</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="13" t="n">
+    <row r="19" ht="25" customHeight="1">
+      <c r="A19" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>TC-T08</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
+      <c r="C19" s="16" t="inlineStr">
         <is>
           <t>管理者</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>先生による送迎取消操作</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t>未完了送迎あり</t>
         </is>
       </c>
-      <c r="F19" s="14" t="inlineStr">
+      <c r="F19" s="17" t="inlineStr">
         <is>
           <t>スケジュール一覧の「取消」ボタンをクリック</t>
         </is>
       </c>
-      <c r="G19" s="14" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
         <is>
           <t>ステータスがキャンセルに変更され、チケット残数は減算されない</t>
         </is>
       </c>
-      <c r="H19" s="15" t="inlineStr">
+      <c r="H19" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I19" s="13" t="inlineStr">
+      <c r="I19" s="16" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J19" s="16" t="inlineStr">
+      <c r="J19" s="19" t="inlineStr">
         <is>
           <t>TC-T08_teacher_cancel.png</t>
         </is>
       </c>
-      <c r="K19" s="14" t="inlineStr">
+      <c r="K19" s="17" t="inlineStr">
         <is>
           <t>先生画面における送迎取消・ステータス管理機能の正常性を確認。</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="17" t="n">
+    <row r="20" ht="25" customHeight="1">
+      <c r="A20" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="B20" s="20" t="inlineStr">
         <is>
           <t>TC-I01</t>
         </is>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
         <is>
           <t>データ整合性</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>エンドツーエンド結合（予約〜完了）</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="E20" s="21" t="inlineStr">
         <is>
           <t>生徒A（残高5回）</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F20" s="21" t="inlineStr">
         <is>
           <t>保護者予約 ➡️ 先生画面で確認 ➡️ 送迎完了 ➡️ 保護者画面確認</t>
         </is>
       </c>
-      <c r="G20" s="18" t="inlineStr">
+      <c r="G20" s="21" t="inlineStr">
         <is>
           <t>生徒Aの残高が4回になり、予約中から完了履歴へ正しく遷移する</t>
         </is>
       </c>
-      <c r="H20" s="15" t="inlineStr">
+      <c r="H20" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I20" s="17" t="inlineStr">
+      <c r="I20" s="20" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J20" s="19" t="inlineStr">
+      <c r="J20" s="22" t="inlineStr">
         <is>
           <t>TC-I01_e2e_integration.png</t>
         </is>
       </c>
-      <c r="K20" s="18" t="inlineStr">
+      <c r="K20" s="21" t="inlineStr">
         <is>
           <t>保護者と管理者の双方向データ連動およびチケット減算の整合性を確認。</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="13" t="n">
+    <row r="21" ht="25" customHeight="1">
+      <c r="A21" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>TC-I02</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>データ整合性</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>残数境界値テスト（アラート〜解除）</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>生徒B（残高1回）</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="F21" s="17" t="inlineStr">
         <is>
           <t>送迎完了(残0:アラート発生) ➡️ 5回券チャージ(残5:アラート解除)</t>
         </is>
       </c>
-      <c r="G21" s="14" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>残数ゼロで黄色警告が表示され、チャージ完了で即座に警告解除される</t>
         </is>
       </c>
-      <c r="H21" s="15" t="inlineStr">
+      <c r="H21" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I21" s="13" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J21" s="16" t="inlineStr">
+      <c r="J21" s="19" t="inlineStr">
         <is>
           <t>TC-I02_boundary_alert_clear.png</t>
         </is>
       </c>
-      <c r="K21" s="14" t="inlineStr">
+      <c r="K21" s="17" t="inlineStr">
         <is>
           <t>残1回での警告表示およびチケット追加時の動的更新を確認。</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="17" t="n">
+    <row r="22" ht="25" customHeight="1">
+      <c r="A22" s="20" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>TC-I03</t>
         </is>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>データ整合性</t>
         </is>
       </c>
-      <c r="D22" s="18" t="inlineStr">
+      <c r="D22" s="21" t="inlineStr">
         <is>
           <t>リロード時のデータ永続化</t>
         </is>
       </c>
-      <c r="E22" s="18" t="inlineStr">
+      <c r="E22" s="21" t="inlineStr">
         <is>
           <t>操作実行済み</t>
         </is>
       </c>
-      <c r="F22" s="18" t="inlineStr">
+      <c r="F22" s="21" t="inlineStr">
         <is>
           <t>ブラウザでCtrl+F5ハードリロードを実施</t>
         </is>
       </c>
-      <c r="G22" s="18" t="inlineStr">
+      <c r="G22" s="21" t="inlineStr">
         <is>
           <t>登録した予約、残数減算、チャージ情報が消えずに維持される</t>
         </is>
       </c>
-      <c r="H22" s="15" t="inlineStr">
+      <c r="H22" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I22" s="17" t="inlineStr">
+      <c r="I22" s="20" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J22" s="19" t="inlineStr">
+      <c r="J22" s="22" t="inlineStr">
         <is>
           <t>TC-I03_reload_persistence.png</t>
         </is>
       </c>
-      <c r="K22" s="18" t="inlineStr">
+      <c r="K22" s="21" t="inlineStr">
         <is>
           <t>ブラウザリロード後も登録データ・チケット情報がLocalStorageに正常保持されることを確認。</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="13" t="n">
+    <row r="23" ht="25" customHeight="1">
+      <c r="A23" s="16" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>TC-U01</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>レスポンシブ</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>スマホ画面幅(375px)レスポンシブ適合</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>iPhone幅</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>375×812 viewportで全画面描画</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="inlineStr">
+        <is>
+          <t>横スクロールなし、タブが下部または適正配置、ボタンタップ領域44px以上</t>
+        </is>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>Puppeteer E2E</t>
+        </is>
+      </c>
+      <c r="J23" s="19" t="inlineStr">
+        <is>
+          <t>TC-U01_mobile_responsive.png</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>iPhoneサイズ（375×812）における横スクロールなし・タップ領域44px以上の適合を確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="25" customHeight="1">
+      <c r="A24" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>TC-V01</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>ビジュアル</t>
+        </is>
+      </c>
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>全画面デザイン・ビジュアル品質検証</t>
+        </is>
+      </c>
+      <c r="E24" s="21" t="inlineStr">
+        <is>
+          <t>PC/スマホ</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="inlineStr">
+        <is>
+          <t>全10画面×PC/スマホ(計20枚)のビジュアル検証</t>
+        </is>
+      </c>
+      <c r="G24" s="21" t="inlineStr">
+        <is>
+          <t>余白・フォント・コントラスト・チップ選択状態が崩れず美しい品質を維持</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" s="20" t="inlineStr">
+        <is>
+          <t>Puppeteer E2E</t>
+        </is>
+      </c>
+      <c r="J24" s="22" t="inlineStr">
+        <is>
+          <t>TC-V01_visual_quality.png</t>
+        </is>
+      </c>
+      <c r="K24" s="21" t="inlineStr">
+        <is>
+          <t>デスクトップ（1280×800）およびモバイル（375×812）における全画面ビジュアル品質・コントラスト・余白の適合を確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="25" customHeight="1">
+      <c r="A25" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
         <is>
           <t>TC-G01</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="C25" s="16" t="inlineStr">
         <is>
           <t>Google連携</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>GASコード表示とワンクリックコピー</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E25" s="17" t="inlineStr">
         <is>
           <t>設定画面</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr">
+      <c r="F25" s="17" t="inlineStr">
         <is>
           <t>「スクリプトをコピー」をクリック</t>
         </is>
       </c>
-      <c r="G23" s="14" t="inlineStr">
+      <c r="G25" s="17" t="inlineStr">
         <is>
           <t>クリップボードにGASスクリプト全文が正確にコピーされる</t>
         </is>
       </c>
-      <c r="H23" s="15" t="inlineStr">
+      <c r="H25" s="23" t="inlineStr">
+        <is>
+          <t>手動受入検証待ち</t>
+        </is>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>手動 (Step 1)</t>
+        </is>
+      </c>
+      <c r="J25" s="19" t="inlineStr">
+        <is>
+          <t>TC-G01_gas_code_view.png</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="inlineStr">
+        <is>
+          <t>Web画面でのコード表示・コピーは自動確認済。Apps Scriptへの貼り付けを手動確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="25" customHeight="1">
+      <c r="A26" s="20" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>TC-G02</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>Google連携</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>シート自動初期化ロジック検証</t>
+        </is>
+      </c>
+      <c r="E26" s="21" t="inlineStr">
+        <is>
+          <t>Googleアカウント</t>
+        </is>
+      </c>
+      <c r="F26" s="21" t="inlineStr">
+        <is>
+          <t>initSpreadsheet関数を実行</t>
+        </is>
+      </c>
+      <c r="G26" s="21" t="inlineStr">
+        <is>
+          <t>生徒台帳・送迎予定履歴・チケット購入履歴の3シートが自動生成される</t>
+        </is>
+      </c>
+      <c r="H26" s="23" t="inlineStr">
+        <is>
+          <t>手動受入検証待ち</t>
+        </is>
+      </c>
+      <c r="I26" s="20" t="inlineStr">
+        <is>
+          <t>手動 (Step 2)</t>
+        </is>
+      </c>
+      <c r="J26" s="24" t="inlineStr">
+        <is>
+          <t>【証跡1】スプレッドシート全景</t>
+        </is>
+      </c>
+      <c r="K26" s="21" t="inlineStr">
+        <is>
+          <t>手動受入手順書Step 2に基づき実施。3シート生成画面のキャプチャー提出でOK。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="25" customHeight="1">
+      <c r="A27" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>TC-G03</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Google連携</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>GAS WebアプリURL設定・保存</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>設定画面</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>設定画面でGAS WebアプリURLを入力し「接続設定を保存」</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>接続先URLがLocalStorageに保存され、緑色フィードバックが表示される</t>
+        </is>
+      </c>
+      <c r="H27" s="23" t="inlineStr">
+        <is>
+          <t>手動受入検証待ち</t>
+        </is>
+      </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>手動 (Step 3)</t>
+        </is>
+      </c>
+      <c r="J27" s="19" t="inlineStr">
+        <is>
+          <t>TC-G03_gas_url_saved.png</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="inlineStr">
+        <is>
+          <t>Web画面でのURL保存機能は自動確認済。発行した実URLの接続テストを手動確認。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="25" customHeight="1">
+      <c r="A28" s="20" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>TC-G04</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>Google連携</t>
+        </is>
+      </c>
+      <c r="D28" s="21" t="inlineStr">
+        <is>
+          <t>Googleカレンダー予定自動登録検証</t>
+        </is>
+      </c>
+      <c r="E28" s="21" t="inlineStr">
+        <is>
+          <t>連携環境</t>
+        </is>
+      </c>
+      <c r="F28" s="21" t="inlineStr">
+        <is>
+          <t>Web画面からテスト予約を登録</t>
+        </is>
+      </c>
+      <c r="G28" s="21" t="inlineStr">
+        <is>
+          <t>Googleカレンダーに『🚗【送迎】生徒名』の予定が自動作成され、シートに行追加される</t>
+        </is>
+      </c>
+      <c r="H28" s="23" t="inlineStr">
+        <is>
+          <t>手動受入検証待ち</t>
+        </is>
+      </c>
+      <c r="I28" s="20" t="inlineStr">
+        <is>
+          <t>手動 (Step 4)</t>
+        </is>
+      </c>
+      <c r="J28" s="24" t="inlineStr">
+        <is>
+          <t>【証跡2&amp;3】シート行追加＆カレンダー</t>
+        </is>
+      </c>
+      <c r="K28" s="21" t="inlineStr">
+        <is>
+          <t>手動受入手順書Step 4に基づき実施。カレンダーおよびシート行追加キャプチャーでOK。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="25" customHeight="1">
+      <c r="A29" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>TC-G05</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>Google連携</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>Googleカレンダー予定自動削除検証</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>連携環境</t>
+        </is>
+      </c>
+      <c r="F29" s="17" t="inlineStr">
+        <is>
+          <t>Web画面からテスト予約をキャンセル</t>
+        </is>
+      </c>
+      <c r="G29" s="17" t="inlineStr">
+        <is>
+          <t>Googleカレンダーの該当送迎予定が自動削除され、シートがcancelledになる</t>
+        </is>
+      </c>
+      <c r="H29" s="23" t="inlineStr">
+        <is>
+          <t>手動受入検証待ち</t>
+        </is>
+      </c>
+      <c r="I29" s="16" t="inlineStr">
+        <is>
+          <t>手動 (Step 5)</t>
+        </is>
+      </c>
+      <c r="J29" s="25" t="inlineStr">
+        <is>
+          <t>【証跡4】カレンダー消去＆cancelled</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="inlineStr">
+        <is>
+          <t>手動受入手順書Step 5に基づき実施。予定削除後の画面キャプチャー提出でOK。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="25" customHeight="1">
+      <c r="A30" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>TC-G06</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>Google連携</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>GAS通信失敗時の自動フォールバック</t>
+        </is>
+      </c>
+      <c r="E30" s="21" t="inlineStr">
+        <is>
+          <t>オフライン/異常系</t>
+        </is>
+      </c>
+      <c r="F30" s="21" t="inlineStr">
+        <is>
+          <t>GAS未デプロイ状態で画面操作を実施</t>
+        </is>
+      </c>
+      <c r="G30" s="21" t="inlineStr">
+        <is>
+          <t>アプリが停止せず、LocalStorageに自動フォールバックして動作継続する</t>
+        </is>
+      </c>
+      <c r="H30" s="18" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I23" s="13" t="inlineStr">
+      <c r="I30" s="20" t="inlineStr">
         <is>
           <t>Puppeteer E2E</t>
         </is>
       </c>
-      <c r="J23" s="16" t="inlineStr">
-        <is>
-          <t>TC-G01_gas_code_view.png</t>
-        </is>
-      </c>
-      <c r="K23" s="14" t="inlineStr">
-        <is>
-          <t>GASバックエンドスクリプト表示およびワンクリックコピーボタンの存在を確認。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="17" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" s="17" t="inlineStr">
-        <is>
-          <t>TC-G02</t>
-        </is>
-      </c>
-      <c r="C24" s="17" t="inlineStr">
-        <is>
-          <t>Google連携</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>シート自動初期化ロジック検証</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>GASコード内</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>initSpreadsheet関数ロジックを検証</t>
-        </is>
-      </c>
-      <c r="G24" s="18" t="inlineStr">
-        <is>
-          <t>生徒台帳・送迎予定履歴・チケット購入履歴の3シート自動生成定義を確認</t>
-        </is>
-      </c>
-      <c r="H24" s="15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" s="17" t="inlineStr">
-        <is>
-          <t>Puppeteer E2E</t>
-        </is>
-      </c>
-      <c r="J24" s="19" t="inlineStr">
-        <is>
-          <t>TC-G02_init_sheets_logic.png</t>
-        </is>
-      </c>
-      <c r="K24" s="18" t="inlineStr">
-        <is>
-          <t>GASスクリプト内に3シート自動初期化関数（initSpreadsheet）が定義されていることを確認。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="13" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>TC-G03</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>Google連携</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>GAS WebアプリURL設定・保存</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>設定画面</t>
-        </is>
-      </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>設定画面でGAS WebアプリURLを入力し「接続設定を保存」</t>
-        </is>
-      </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>接続先URLがLocalStorageに保存され、緑色フィードバックが表示される</t>
-        </is>
-      </c>
-      <c r="H25" s="15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" s="13" t="inlineStr">
-        <is>
-          <t>Puppeteer E2E</t>
-        </is>
-      </c>
-      <c r="J25" s="16" t="inlineStr">
-        <is>
-          <t>TC-G03_gas_url_saved.png</t>
-        </is>
-      </c>
-      <c r="K25" s="14" t="inlineStr">
-        <is>
-          <t>GAS WebアプリURLの入力およびLocalStorage保存フィードバックを確認。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t>TC-G04</t>
-        </is>
-      </c>
-      <c r="C26" s="17" t="inlineStr">
-        <is>
-          <t>Google連携</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Googleカレンダー予定自動登録検証</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>連携仕様</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>GAS内のCalendarApp連携ロジックを検証</t>
-        </is>
-      </c>
-      <c r="G26" s="18" t="inlineStr">
-        <is>
-          <t>Googleカレンダーに『🚗【送迎】生徒名』の予定が自動作成される定義を確認</t>
-        </is>
-      </c>
-      <c r="H26" s="15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" s="17" t="inlineStr">
-        <is>
-          <t>Puppeteer E2E</t>
-        </is>
-      </c>
-      <c r="J26" s="19" t="inlineStr">
-        <is>
-          <t>TC-G04_calendar_sync_logic.png</t>
-        </is>
-      </c>
-      <c r="K26" s="18" t="inlineStr">
-        <is>
-          <t>GASコード内にCalendarApp.createEventによる『🚗【送迎】生徒名』の自動登録ロジックを確認。</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="13" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>TC-G05</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>Google連携</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>Googleカレンダー予定自動削除検証</t>
-        </is>
-      </c>
-      <c r="E27" s="14" t="inlineStr">
-        <is>
-          <t>連携仕様</t>
-        </is>
-      </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>GAS内のcancelReservationロジックを検証</t>
-        </is>
-      </c>
-      <c r="G27" s="14" t="inlineStr">
-        <is>
-          <t>Googleカレンダーの該当送迎予定がdeleteEvent()で自動削除される定義を確認</t>
-        </is>
-      </c>
-      <c r="H27" s="15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" s="13" t="inlineStr">
-        <is>
-          <t>Puppeteer E2E</t>
-        </is>
-      </c>
-      <c r="J27" s="16" t="inlineStr">
-        <is>
-          <t>TC-G05_calendar_delete_logic.png</t>
-        </is>
-      </c>
-      <c r="K27" s="14" t="inlineStr">
-        <is>
-          <t>GASコード内にキャンセル時のGoogleカレンダー自動削除ロジック（deleteEvent）を確認。</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="17" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>TC-G06</t>
-        </is>
-      </c>
-      <c r="C28" s="17" t="inlineStr">
-        <is>
-          <t>Google連携</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
-        <is>
-          <t>GAS通信失敗時の自動フォールバック</t>
-        </is>
-      </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>オフライン/異常系</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>GAS未デプロイ状態で画面操作を実施</t>
-        </is>
-      </c>
-      <c r="G28" s="18" t="inlineStr">
-        <is>
-          <t>アプリが停止せず、LocalStorageに自動フォールバックして動作継続する</t>
-        </is>
-      </c>
-      <c r="H28" s="15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" s="17" t="inlineStr">
-        <is>
-          <t>Puppeteer E2E</t>
-        </is>
-      </c>
-      <c r="J28" s="19" t="inlineStr">
+      <c r="J30" s="22" t="inlineStr">
         <is>
           <t>TC-G06_fallback_handling.png</t>
         </is>
       </c>
-      <c r="K28" s="18" t="inlineStr">
-        <is>
-          <t>GAS未接続・オフライン時もLocalStorageフォールバックにより動作継続することを確認。</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="13" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>TC-U01</t>
-        </is>
-      </c>
-      <c r="C29" s="13" t="inlineStr">
-        <is>
-          <t>レスポンシブ</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>スマホ画面幅(375px)レスポンシブ適合</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="inlineStr">
-        <is>
-          <t>iPhone幅</t>
-        </is>
-      </c>
-      <c r="F29" s="14" t="inlineStr">
-        <is>
-          <t>375×812 viewportで全画面描画</t>
-        </is>
-      </c>
-      <c r="G29" s="14" t="inlineStr">
-        <is>
-          <t>横スクロールなし、タブが下部または適正配置、ボタンタップ領域44px以上</t>
-        </is>
-      </c>
-      <c r="H29" s="15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" s="13" t="inlineStr">
-        <is>
-          <t>Puppeteer E2E</t>
-        </is>
-      </c>
-      <c r="J29" s="16" t="inlineStr">
-        <is>
-          <t>TC-U01_mobile_responsive.png</t>
-        </is>
-      </c>
-      <c r="K29" s="14" t="inlineStr">
-        <is>
-          <t>iPhoneサイズ（375×812）における横スクロールなし・タップ領域44px以上の適合を確認。</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="17" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" s="17" t="inlineStr">
-        <is>
-          <t>TC-V01</t>
-        </is>
-      </c>
-      <c r="C30" s="17" t="inlineStr">
-        <is>
-          <t>ビジュアル</t>
-        </is>
-      </c>
-      <c r="D30" s="18" t="inlineStr">
-        <is>
-          <t>全画面デザイン・ビジュアル品質検証</t>
-        </is>
-      </c>
-      <c r="E30" s="18" t="inlineStr">
-        <is>
-          <t>PC/スマホ</t>
-        </is>
-      </c>
-      <c r="F30" s="18" t="inlineStr">
-        <is>
-          <t>全10画面×PC/スマホ(計20枚)のビジュアル検証</t>
-        </is>
-      </c>
-      <c r="G30" s="18" t="inlineStr">
-        <is>
-          <t>余白・フォント・コントラスト・チップ選択状態が崩れず美しい品質を維持</t>
-        </is>
-      </c>
-      <c r="H30" s="15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" s="17" t="inlineStr">
-        <is>
-          <t>Puppeteer E2E</t>
-        </is>
-      </c>
-      <c r="J30" s="19" t="inlineStr">
-        <is>
-          <t>TC-V01_visual_quality.png</t>
-        </is>
-      </c>
-      <c r="K30" s="18" t="inlineStr">
-        <is>
-          <t>デスクトップ（1280×800）およびモバイル（375×812）における全画面ビジュアル品質・コントラスト・余白の適合を確認。</t>
+      <c r="K30" s="21" t="inlineStr">
+        <is>
+          <t>自動E2E検証完了。GAS未接続時もFail-Openにより画面操作が停止しないことを実証済。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:E23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Google連携（スプレッドシート＆カレンダー）手動受入検証 手順＆証跡貼付表</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>※技術的知識のない方でも本手順を実施し、各証跡画像を添付・確認することで正式合格（Pass）となります</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>ステップ</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>実施項目</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>具体的な操作手順（迷わずできる手順）</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>合格に必要な証跡</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Step 1</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>スプレッドシート作成 &amp; コード貼付</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>Googleドライブで「空白のスプレッドシート」を作成 ➜ メニュー「拡張機能」&gt;「Apps Script」 ➜ Webアプリ「Google連携」タブの「スクリプトをコピー」を押してエディタに貼り付け ➜ 保存</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="inlineStr">
+        <is>
+          <t>スクリプト保存完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Step 2</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>3シート自動初期化 &amp; アクセス承認</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>プルダウンで「initSpreadsheet」を選択し「実行」 ➜ 「権限を確認」 ➜ 「詳細」&gt;「安全ではないページに移動」&gt;「許可」 ➜ スプレッドシート下に3シート（生徒台帳、送迎予定履歴、チケット購入履歴）が生成される</t>
+        </is>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>【証跡1】3シート生成画面キャプチャー</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Step 3</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>Webアプリデプロイ &amp; URL連携</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>右上の「デプロイ」&gt;「新しいデプロイ」 ➜ 種類「ウェブアプリ」、アクセス「全員」でデプロイ ➜ 表示されたURLをコピー ➜ Webアプリ「Google連携」タブに貼り付けて「接続設定を保存」</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="inlineStr">
+        <is>
+          <t>URL保存完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>Step 4</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>テスト予約登録 &amp; カレンダー・シート確認</t>
+        </is>
+      </c>
+      <c r="D9" s="32" t="inlineStr">
+        <is>
+          <t>Webアプリ「送迎利用者用」で山本颯太くんを選択 ➜ 「送迎の予約を申し込む」（送迎日、16:30、行き、メモ:テスト） ➜ スプレッドシート「送迎予定履歴」に行追加 &amp; Googleカレンダーに『🚗【送迎】山本 颯太』登録を確認</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>【証跡2&amp;3】シート行追加 &amp; カレンダー予定キャプチャー</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Step 5</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>キャンセル連動 &amp; カレンダー自動削除</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>Webアプリでテスト予約の「キャンセル」をクリック ➜ Googleカレンダーから予定が自動消去されたことを確認 ➜ スプレッドシートのステータスが「cancelled」に自動更新されたことを確認</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="inlineStr">
+        <is>
+          <t>【証跡4】予定消去 &amp; cancelled更新キャプチャー</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>▍手動受入検証 証跡キャプチャー貼付 ＆ 受入サイン欄</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>検証証跡 1: シート自動生成画面</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>スプレッドシート下部に「生徒台帳」「送迎予定履歴」「チケット購入履歴」の3シートが表示されている画面</t>
+        </is>
+      </c>
+      <c r="D15" s="34" t="inlineStr">
+        <is>
+          <t>[   ] 確認完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>検証証跡 2: スプレッドシート行追加画面</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>「送迎予定履歴」シートに、Webアプリから登録したテスト予約（16:30 行き）が追加されている画面</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="inlineStr">
+        <is>
+          <t>[   ] 確認完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>検証証跡 3: Googleカレンダー予定自動登録</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Googleカレンダーの該当日時に『🚗【送迎】生徒名』の予定が自動登録されている画面</t>
+        </is>
+      </c>
+      <c r="D17" s="34" t="inlineStr">
+        <is>
+          <t>[   ] 確認完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>検証証跡 4: カレンダー予定削除 &amp; cancelled更新</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Webアプリでキャンセル後、カレンダー予定が消え、シートステータスが「cancelled」になった画面</t>
+        </is>
+      </c>
+      <c r="D18" s="34" t="inlineStr">
+        <is>
+          <t>[   ] 確認完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>検証実施日: 2026年 _____月 _____日</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="35" t="inlineStr">
+        <is>
+          <t>検証実施者ご署名: _______________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="35" t="inlineStr">
+        <is>
+          <t>使用Googleアカウント: _______________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="36" t="inlineStr">
+        <is>
+          <t>総合受入判定: [   ] 合格（本番リリース承認）   /   [   ] 不合格（再調整要）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: specify verification account k-umezawa@ml-mightylink.com in manual UAT guide and test spec
</commit_message>
<xml_diff>
--- a/docs/GoogleDrive_Upload/Mauro_Brenda_Taxi_Link_シナリオテスト仕様書.xlsx
+++ b/docs/GoogleDrive_Upload/Mauro_Brenda_Taxi_Link_シナリオテスト仕様書.xlsx
@@ -2839,21 +2839,21 @@
     <row r="20">
       <c r="B20" s="35" t="inlineStr">
         <is>
-          <t>検証実施日: 2026年 _____月 _____日</t>
+          <t>検証実施日: 2026年 10月 _____日</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="35" t="inlineStr">
         <is>
-          <t>検証実施者ご署名: _______________________________</t>
+          <t>検証実施者ご署名: 梅澤 研太 様 (または検証ご担当者様)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="35" t="inlineStr">
         <is>
-          <t>使用Googleアカウント: _______________________________</t>
+          <t>使用Googleアカウント: k-umezawa@ml-mightylink.com</t>
         </is>
       </c>
     </row>

</xml_diff>